<commit_message>
Minor changes to grid
Changed the EEZ and state name attribute for a hand full of grid cells on the periphery and intersecting the EEZ
</commit_message>
<xml_diff>
--- a/spatial_data/grids/ten arcminute grid polys shore METADATA.xlsx
+++ b/spatial_data/grids/ten arcminute grid polys shore METADATA.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10913"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/blake.feist/Documents/GitHub/VMS-pipeline/spatial_data/grids/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA538339-A4A6-C141-8B0A-147B8C3665CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B50B00AD-887F-B14D-9DE8-E8EDCE6E373A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" activeTab="1" xr2:uid="{AD14FED6-09D0-AC4E-9FD4-5D358E8F4B1E}"/>
   </bookViews>
@@ -113,9 +113,6 @@
     <t>Weighted mean depth of grid cell based on Feist et al. bathymetry</t>
   </si>
   <si>
-    <t>Number of Feist et al. bathymetry grid cells within 5km grid cell</t>
-  </si>
-  <si>
     <t>Median depth of grid cell based on Feist et al. bathymetry</t>
   </si>
   <si>
@@ -398,13 +395,16 @@
   <si>
     <t>Not all RAMP zone latitudinal boundaries are at multiples of 10-arcminutes, so some 10-arcminute grid cells are not fully within the listed RAMP zone. 10-arcminute grid cells with "majority" attribute do not share a common border with the associated RAMP zone. However, the majority of the area of that grid cell falls within the corresponding RAMP zone.</t>
   </si>
+  <si>
+    <t>Number of Feist et al. bathymetry grid cells within grid cell</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="[$-409]d\-mmm\-yyyy;@"/>
+    <numFmt numFmtId="164" formatCode="[$-409]d\-mmm\-yyyy;@"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -477,7 +477,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -803,15 +803,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>57</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B2" s="7">
         <v>45919</v>
@@ -819,137 +819,137 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="102" x14ac:dyDescent="0.2">
       <c r="A4" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B8" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B11" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B13" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B14" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B15" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B16" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B17" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B18" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B20" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B21" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B22" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B23" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B24" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B25" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B26" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B27" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="51" x14ac:dyDescent="0.2">
       <c r="A28" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -995,7 +995,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>18</v>
@@ -1008,10 +1008,10 @@
     </row>
     <row r="3" spans="1:6" s="2" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>13</v>
@@ -1022,10 +1022,10 @@
     </row>
     <row r="4" spans="1:6" s="2" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>23</v>
@@ -1036,25 +1036,25 @@
     </row>
     <row r="5" spans="1:6" s="2" customFormat="1" ht="85" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" s="2" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" s="2" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>23</v>
@@ -1067,7 +1067,7 @@
         <v>8</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>19</v>
@@ -1076,7 +1076,7 @@
         <v>17</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>22</v>
@@ -1084,10 +1084,10 @@
     </row>
     <row r="8" spans="1:6" s="2" customFormat="1" ht="68" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>19</v>
@@ -1096,7 +1096,7 @@
         <v>16</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F8" s="3"/>
     </row>
@@ -1105,67 +1105,67 @@
         <v>9</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F9" s="3"/>
     </row>
-    <row r="10" spans="1:6" s="2" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" s="2" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>23</v>
       </c>
       <c r="D10" s="3"/>
       <c r="E10" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F10" s="3"/>
     </row>
     <row r="11" spans="1:6" s="2" customFormat="1" ht="136" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>13</v>
       </c>
       <c r="D11" s="3"/>
       <c r="E11" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12" spans="1:6" s="2" customFormat="1" ht="85" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>13</v>
       </c>
       <c r="D12" s="3"/>
       <c r="E12" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="13" spans="1:6" s="2" customFormat="1" ht="34" x14ac:dyDescent="0.2">
@@ -1180,7 +1180,7 @@
       </c>
       <c r="D13" s="3"/>
       <c r="F13" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="14" spans="1:6" s="2" customFormat="1" ht="34" x14ac:dyDescent="0.2">
@@ -1188,14 +1188,14 @@
         <v>2</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>25</v>
+        <v>117</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>19</v>
       </c>
       <c r="D14" s="3"/>
       <c r="F14" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="15" spans="1:6" s="2" customFormat="1" ht="34" x14ac:dyDescent="0.2">
@@ -1203,7 +1203,7 @@
         <v>3</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>23</v>
@@ -1211,7 +1211,7 @@
       <c r="D15" s="3"/>
       <c r="E15" s="3"/>
       <c r="F15" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="16" spans="1:6" s="2" customFormat="1" ht="34" x14ac:dyDescent="0.2">
@@ -1219,14 +1219,14 @@
         <v>4</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>23</v>
       </c>
       <c r="D16" s="3"/>
       <c r="F16" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="17" spans="1:6" s="2" customFormat="1" ht="34" x14ac:dyDescent="0.2">
@@ -1234,7 +1234,7 @@
         <v>5</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>23</v>
@@ -1242,7 +1242,7 @@
       <c r="D17" s="3"/>
       <c r="E17" s="3"/>
       <c r="F17" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="18" spans="1:6" s="2" customFormat="1" ht="34" x14ac:dyDescent="0.2">
@@ -1250,7 +1250,7 @@
         <v>6</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>23</v>
@@ -1258,7 +1258,7 @@
       <c r="D18" s="3"/>
       <c r="E18" s="3"/>
       <c r="F18" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="19" spans="1:6" s="2" customFormat="1" ht="34" x14ac:dyDescent="0.2">
@@ -1266,7 +1266,7 @@
         <v>7</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>23</v>
@@ -1274,18 +1274,18 @@
       <c r="D19" s="3"/>
       <c r="E19" s="3"/>
       <c r="F19" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="20" spans="1:6" s="2" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D20" s="3"/>
       <c r="E20" s="3"/>
@@ -1293,10 +1293,10 @@
     </row>
     <row r="21" spans="1:6" s="2" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>13</v>
@@ -1307,10 +1307,10 @@
     </row>
     <row r="22" spans="1:6" s="2" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>13</v>
@@ -1321,10 +1321,10 @@
     </row>
     <row r="23" spans="1:6" s="2" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>13</v>
@@ -1335,10 +1335,10 @@
     </row>
     <row r="24" spans="1:6" s="2" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>13</v>
@@ -1349,10 +1349,10 @@
     </row>
     <row r="25" spans="1:6" s="2" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>13</v>
@@ -1363,10 +1363,10 @@
     </row>
     <row r="26" spans="1:6" s="2" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>13</v>
@@ -1377,10 +1377,10 @@
     </row>
     <row r="27" spans="1:6" s="2" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>13</v>
@@ -1391,10 +1391,10 @@
     </row>
     <row r="28" spans="1:6" s="2" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>13</v>
@@ -1405,39 +1405,39 @@
     </row>
     <row r="29" spans="1:6" s="2" customFormat="1" ht="136" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="E29" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="E29" s="3" t="s">
+      <c r="F29" s="3" t="s">
         <v>111</v>
-      </c>
-      <c r="F29" s="3" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="30" spans="1:6" s="2" customFormat="1" ht="102" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B30" s="3" t="s">
         <v>115</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>116</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>19</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F30" s="3"/>
     </row>

</xml_diff>